<commit_message>
Solve failing RPA tests.
</commit_message>
<xml_diff>
--- a/DocumentUnderstandingProcess/contentFiles/any/any/pt0/VisualBasic/Tests/Cache/ExportMergedDocuments_1-1.xlsx
+++ b/DocumentUnderstandingProcess/contentFiles/any/any/pt0/VisualBasic/Tests/Cache/ExportMergedDocuments_1-1.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
     <x:t>File Number</x:t>
   </x:si>
@@ -33,6 +33,9 @@
   </x:si>
   <x:si>
     <x:t>11/12/2009</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Texas</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -410,6 +413,9 @@
       <x:c r="C2" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -452,6 +458,9 @@
       <x:c r="C2" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>

</xml_diff>